<commit_message>
Results for Model 4 have been fixed successfully
</commit_message>
<xml_diff>
--- a/Hypothesis_check.xlsx
+++ b/Hypothesis_check.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\KILB\Ziay\HiWi\Warrier\02_OUTPUT\Files\Altair Repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0954BF4-ECB3-4F39-88A2-93D8FE2238F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3550C95F-B745-484C-804D-6A7F3E5EF3A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{4621E9A4-ED71-4947-ABCD-86ECFC03C30D}"/>
   </bookViews>
@@ -180,7 +180,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -195,22 +195,40 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -348,53 +366,25 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -416,27 +406,29 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Schlecht" xfId="1" builtinId="27"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Zelle überprüfen" xfId="2" builtinId="23"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -449,6 +441,99 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>409575</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>738818</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Grafik 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26007E24-FDCB-9F15-C410-350E32B83BB1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6972300" y="5267325"/>
+          <a:ext cx="7187243" cy="4514850"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>409576</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>200025</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9526</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>161810</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Grafik 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9674A56-55F7-9EB5-137C-9DB45AFA4D69}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6972301" y="200025"/>
+          <a:ext cx="7219950" cy="4905260"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -768,1076 +853,1079 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{777E7DAB-147F-49EF-81FC-E47C0F5DE28B}">
-  <dimension ref="A1:G46"/>
+  <dimension ref="B1:H47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="17.5703125" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.28515625" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" customWidth="1"/>
     <col min="6" max="6" width="13.5703125" customWidth="1"/>
     <col min="7" max="7" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="2:8" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="C2" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D2" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="E2" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="F2" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="G2" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="H2" s="8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="7">
+    <row r="3" spans="2:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="12">
         <v>1</v>
       </c>
-      <c r="B2" s="8">
+      <c r="C3" s="7">
         <v>1</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" s="8" t="s">
+      <c r="D3" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="E3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B4" s="11">
         <v>1</v>
       </c>
-      <c r="B3" s="1">
+      <c r="C4" s="1">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="D4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H4" s="10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="11">
         <v>1</v>
       </c>
-      <c r="B4" s="1">
+      <c r="C5" s="1">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="D5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H5" s="10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="2">
         <v>1</v>
       </c>
-      <c r="B5" s="1">
+      <c r="C6" s="1">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>1</v>
-      </c>
-      <c r="B6" s="1">
-        <v>5</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="D6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="G6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="2">
         <v>1</v>
       </c>
-      <c r="B7" s="1">
+      <c r="C7" s="1">
+        <v>5</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1">
         <v>6</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="G8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+      <c r="H8" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="11">
         <v>2</v>
       </c>
-      <c r="B8" s="1">
+      <c r="C9" s="1">
         <v>1</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="D9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H9" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="11">
         <v>2</v>
       </c>
-      <c r="B9" s="1">
+      <c r="C10" s="1">
         <v>2</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="D10" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H10" s="10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="11">
         <v>2</v>
       </c>
-      <c r="B10" s="1">
+      <c r="C11" s="1">
         <v>3</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" s="1" t="s">
+      <c r="D11" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="G11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H11" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="2">
         <v>2</v>
       </c>
-      <c r="B11" s="1">
+      <c r="C12" s="1">
         <v>4</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="D12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G11" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+      <c r="H12" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="2">
         <v>2</v>
       </c>
-      <c r="B12" s="1">
+      <c r="C13" s="1">
         <v>5</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="D13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+      <c r="H13" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="2">
         <v>2</v>
       </c>
-      <c r="B13" s="1">
+      <c r="C14" s="1">
         <v>6</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E13" s="1" t="s">
+      <c r="D14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="G14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+      <c r="H14" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B15" s="2">
         <v>3</v>
       </c>
-      <c r="B14" s="1">
+      <c r="C15" s="1">
         <v>1</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D14" s="1" t="s">
+      <c r="D15" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="G15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H15" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+    <row r="16" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B16" s="2">
         <v>3</v>
       </c>
-      <c r="B15" s="1">
+      <c r="C16" s="1">
         <v>2</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D15" s="1" t="s">
+      <c r="D16" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="G16" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+    <row r="17" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B17" s="2">
         <v>3</v>
       </c>
-      <c r="B16" s="1">
+      <c r="C17" s="1">
         <v>3</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D16" s="1" t="s">
+      <c r="D17" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E17" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="G17" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H17" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="2">
         <v>3</v>
       </c>
-      <c r="B17" s="1">
+      <c r="C18" s="1">
         <v>4</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E17" s="1" t="s">
+      <c r="D18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="G18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G17" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+      <c r="H18" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B19" s="2">
         <v>3</v>
       </c>
-      <c r="B18" s="1">
+      <c r="C19" s="1">
         <v>5</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E18" s="1" t="s">
+      <c r="D19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="G19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G18" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+      <c r="H19" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="2">
         <v>3</v>
       </c>
-      <c r="B19" s="1">
+      <c r="C20" s="1">
         <v>6</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E19" s="1" t="s">
+      <c r="D20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="G20" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+      <c r="H20" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B21" s="2">
         <v>4</v>
       </c>
-      <c r="B20" s="1">
+      <c r="C21" s="1">
         <v>1</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D20" s="1" t="s">
+      <c r="D21" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F20" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="H21" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+    <row r="22" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B22" s="2">
         <v>4</v>
       </c>
-      <c r="B21" s="1">
+      <c r="C22" s="1">
         <v>2</v>
       </c>
-      <c r="C21" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D21" s="1" t="s">
+      <c r="D22" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="F22" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F21" s="1" t="s">
+      <c r="G22" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G21" s="3" t="s">
+      <c r="H22" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+    <row r="23" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B23" s="2">
         <v>4</v>
       </c>
-      <c r="B22" s="1">
+      <c r="C23" s="1">
         <v>3</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D22" s="1" t="s">
+      <c r="D23" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E23" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="G23" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="H23" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B24" s="2">
         <v>4</v>
       </c>
-      <c r="B23" s="1">
+      <c r="C24" s="1">
         <v>4</v>
       </c>
-      <c r="C23" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E23" s="1" t="s">
+      <c r="D24" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="G24" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G23" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+      <c r="H24" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B25" s="2">
         <v>4</v>
       </c>
-      <c r="B24" s="1">
+      <c r="C25" s="1">
         <v>5</v>
       </c>
-      <c r="C24" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E24" s="1" t="s">
+      <c r="D25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F24" s="1" t="s">
+      <c r="G25" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G24" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+      <c r="H25" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B26" s="2">
         <v>4</v>
       </c>
-      <c r="B25" s="1">
+      <c r="C26" s="1">
         <v>6</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E25" s="1" t="s">
+      <c r="D26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="G26" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+      <c r="H26" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B27" s="2">
         <v>5</v>
       </c>
-      <c r="B26" s="1">
+      <c r="C27" s="1">
         <v>1</v>
       </c>
-      <c r="C26" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D26" s="1" t="s">
+      <c r="D27" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E27" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="F27" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="1" t="s">
+      <c r="G27" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G26" s="3" t="s">
+      <c r="H27" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
+    <row r="28" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B28" s="2">
         <v>5</v>
       </c>
-      <c r="B27" s="1">
+      <c r="C28" s="1">
         <v>2</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D27" s="1" t="s">
+      <c r="D28" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E28" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="F28" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="G28" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="H28" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+    <row r="29" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B29" s="2">
         <v>5</v>
       </c>
-      <c r="B28" s="1">
+      <c r="C29" s="1">
         <v>3</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D28" s="1" t="s">
+      <c r="D29" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E29" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="G29" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G28" s="3" t="s">
+      <c r="H29" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B30" s="2">
         <v>5</v>
       </c>
-      <c r="B29" s="1">
+      <c r="C30" s="1">
         <v>4</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E29" s="1" t="s">
+      <c r="D30" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F29" s="1" t="s">
+      <c r="G30" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G29" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+      <c r="H30" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B31" s="2">
         <v>5</v>
       </c>
-      <c r="B30" s="1">
+      <c r="C31" s="1">
         <v>5</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E30" s="1" t="s">
+      <c r="D31" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="G31" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G30" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
+      <c r="H31" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B32" s="2">
         <v>5</v>
       </c>
-      <c r="B31" s="1">
+      <c r="C32" s="1">
         <v>6</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" s="1" t="s">
+      <c r="D32" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="G32" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G31" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
+      <c r="H32" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B33" s="2">
         <v>6</v>
       </c>
-      <c r="B32" s="1">
+      <c r="C33" s="1">
         <v>1</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D32" s="1" t="s">
+      <c r="D33" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E33" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="F33" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F32" s="1" t="s">
+      <c r="G33" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G32" s="3" t="s">
+      <c r="H33" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
+    <row r="34" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B34" s="2">
         <v>6</v>
       </c>
-      <c r="B33" s="1">
+      <c r="C34" s="1">
         <v>2</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D33" s="1" t="s">
+      <c r="D34" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E34" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="F34" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="G34" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G33" s="3" t="s">
+      <c r="H34" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
+    <row r="35" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B35" s="2">
         <v>6</v>
       </c>
-      <c r="B34" s="1">
+      <c r="C35" s="1">
         <v>3</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D34" s="1" t="s">
+      <c r="D35" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E35" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="F35" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F34" s="1" t="s">
+      <c r="G35" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="H35" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B36" s="2">
         <v>6</v>
       </c>
-      <c r="B35" s="1">
+      <c r="C36" s="1">
         <v>4</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E35" s="1" t="s">
+      <c r="D36" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F35" s="1" t="s">
+      <c r="G36" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G35" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+      <c r="H36" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B37" s="2">
         <v>6</v>
       </c>
-      <c r="B36" s="1">
+      <c r="C37" s="1">
         <v>5</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E36" s="1" t="s">
+      <c r="D37" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="G37" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G36" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="2">
+      <c r="H37" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B38" s="2">
         <v>6</v>
       </c>
-      <c r="B37" s="1">
+      <c r="C38" s="1">
         <v>6</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E37" s="1" t="s">
+      <c r="D38" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F37" s="1" t="s">
+      <c r="G38" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G37" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
+      <c r="H38" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B39" s="2">
         <v>7</v>
       </c>
-      <c r="B38" s="1">
+      <c r="C39" s="1">
         <v>1</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D38" s="1" t="s">
+      <c r="D39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E39" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="F39" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F38" s="1" t="s">
+      <c r="G39" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G38" s="3" t="s">
+      <c r="H39" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
+    <row r="40" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B40" s="2">
         <v>7</v>
       </c>
-      <c r="B39" s="1">
+      <c r="C40" s="1">
         <v>2</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D39" s="1" t="s">
+      <c r="D40" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="F40" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="G40" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G39" s="3" t="s">
+      <c r="H40" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
+    <row r="41" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B41" s="2">
         <v>7</v>
       </c>
-      <c r="B40" s="1">
+      <c r="C41" s="1">
         <v>3</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D40" s="1" t="s">
+      <c r="D41" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E41" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="F41" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="G41" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G40" s="3" t="s">
+      <c r="H41" s="3" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B42" s="2">
         <v>7</v>
       </c>
-      <c r="B41" s="1">
+      <c r="C42" s="1">
         <v>4</v>
       </c>
-      <c r="C41" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E41" s="1" t="s">
+      <c r="D42" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="G42" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G41" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
+      <c r="H42" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B43" s="2">
         <v>7</v>
       </c>
-      <c r="B42" s="1">
+      <c r="C43" s="1">
         <v>5</v>
       </c>
-      <c r="C42" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E42" s="1" t="s">
+      <c r="D43" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F42" s="1" t="s">
+      <c r="G43" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="G42" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
+      <c r="H43" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B44" s="2">
         <v>7</v>
       </c>
-      <c r="B43" s="1">
+      <c r="C44" s="1">
         <v>6</v>
       </c>
-      <c r="C43" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E43" s="1" t="s">
+      <c r="D44" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="G44" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G43" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
+      <c r="H44" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B45" s="2">
         <v>8</v>
       </c>
-      <c r="B44" s="1">
+      <c r="C45" s="1">
         <v>1</v>
       </c>
-      <c r="C44" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D44" s="1" t="s">
+      <c r="D45" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E45" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E44" s="1" t="s">
+      <c r="F45" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="G45" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="G44" s="3" t="s">
+      <c r="H45" s="3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
+    <row r="46" spans="2:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B46" s="2">
         <v>8</v>
       </c>
-      <c r="B45" s="1">
+      <c r="C46" s="1">
         <v>2</v>
       </c>
-      <c r="C45" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D45" s="1" t="s">
+      <c r="D46" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E46" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E45" s="1" t="s">
+      <c r="F46" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="F45" s="1" t="s">
+      <c r="G46" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="G45" s="3" t="s">
+      <c r="H46" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="4">
+    <row r="47" spans="2:8" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="4">
         <v>8</v>
       </c>
-      <c r="B46" s="5">
+      <c r="C47" s="5">
         <v>3</v>
       </c>
-      <c r="C46" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="D46" s="5" t="s">
+      <c r="D47" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="E47" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="F47" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F46" s="5" t="s">
+      <c r="G47" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G46" s="6" t="s">
+      <c r="H47" s="6" t="s">
         <v>37</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>